<commit_message>
Parse Type-A monthly summaries and render Hebrew correctly
- Extend the Type-A parser and generator with day of week, working days,
  monthly hours, hourly rate and total payment
- Render Hebrew right-to-left in the generated PDF (python-bidi)
- Improve Type-B parsing, OCR handling and the rules engine
- Narrow the time jitter to ±5 minutes
- Refresh the sample outputs
</commit_message>
<xml_diff>
--- a/samples/a_r_25_out.xlsx
+++ b/samples/a_r_25_out.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -520,7 +520,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>עובד: —    תקופה: 2023-02-07 – 2023-02-26</t>
+          <t>עובד: —    תקופה: 2023-02-01 – 2023-02-27</t>
         </is>
       </c>
     </row>
@@ -590,33 +590,33 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>07/02/2023</t>
+          <t>01/02/2023</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>יום שלישי</t>
+          <t>יום רביעי</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>15.48</t>
+          <t>7.97</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
@@ -625,40 +625,40 @@
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>daily_hours mismatch: declared=7.50 computed=15.50 diff=8.00</t>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>13/02/2023</t>
+          <t>02/02/2023</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>יום שני</t>
+          <t>יום חמישי</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>00:33</t>
+          <t>08:09</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>14.43</t>
+          <t>7.97</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
@@ -667,40 +667,40 @@
       <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>daily_hours mismatch: declared=6.50 computed=14.50 diff=8.00</t>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>14/02/2023</t>
+          <t>05/02/2023</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>יום שלישי</t>
+          <t>יום ראשון</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>00:26</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>15.50</t>
+          <t>8.25</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
@@ -709,40 +709,40 @@
       <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>daily_hours mismatch: declared=7.50 computed=15.50 diff=8.00</t>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>16/02/2023</t>
+          <t>07/02/2023</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>יום חמישי</t>
+          <t>יום שלישי</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>00:39</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>16.33</t>
+          <t>7.87</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
@@ -751,40 +751,40 @@
       <c r="K8" s="4" t="inlineStr"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>daily_hours mismatch: declared=7.50 computed=16.50 diff=9.00</t>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>20/02/2023</t>
+          <t>12/02/2023</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>יום שני</t>
+          <t>יום ראשון</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>00:26</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>15.42</t>
+          <t>8.12</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr"/>
@@ -793,40 +793,40 @@
       <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>daily_hours mismatch: declared=7.50 computed=15.50 diff=8.00</t>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>22/02/2023</t>
+          <t>13/02/2023</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>יום רביעי</t>
+          <t>יום שני</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>00:32</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>14:52</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>15.63</t>
+          <t>6.95</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
@@ -835,40 +835,40 @@
       <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>daily_hours mismatch: declared=7.50 computed=15.50 diff=8.00</t>
+          <t>daily_hours mismatch: declared=6.50 computed=7.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>23/02/2023</t>
+          <t>14/02/2023</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>יום חמישי</t>
+          <t>יום שלישי</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>00:34</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>14.50</t>
+          <t>7.75</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
@@ -877,40 +877,40 @@
       <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>daily_hours mismatch: declared=6.50 computed=14.50 diff=8.00</t>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>26/02/2023</t>
+          <t>15/02/2023</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>יום ראשון</t>
+          <t>יום רביעי</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>00:29</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>8.12</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
@@ -919,113 +919,407 @@
       <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>daily_hours mismatch: declared=7.50 computed=15.50 diff=8.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr"/>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr"/>
-      <c r="E13" s="5" t="inlineStr"/>
-      <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>122.86</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
-      <c r="K13" s="5" t="inlineStr"/>
-      <c r="L13" s="5" t="inlineStr"/>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>16/02/2023</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>יום חמישי</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>7.98</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>19/02/2023</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>יום ראשון</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>7.80</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>ימים</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>8</v>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>20/02/2023</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>יום שני</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>8.22</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>סה"כ שעות</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>122.86</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>22/02/2023</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>יום רביעי</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>08:08</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>7.93</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>100% שעות</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>122.86</t>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>23/02/2023</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>יום חמישי</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>7.05</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>daily_hours mismatch: declared=6.50 computed=7.00 diff=0.50</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>125% שעות</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>0</v>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>26/02/2023</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>יום ראשון</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>07:58</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>16:08</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>8.17</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>150% שעות</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>150% שבת</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>בונוס</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>27/02/2023</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>יום שני</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>7.73</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>117.88</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>ימים</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>סה"כ שעות</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>117.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>100% שעות</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>117.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>125% שעות</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>150% שעות</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>150% שבת</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>בונוס</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
           <t>נסיעות</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B29" s="7" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a README and regenerate the sample outputs
- Describe the tool as a synthetic-data generator, its pipeline, how to
  install Tesseract with Hebrew, run it and run the tests
- Regenerate the sample outputs with the fixed parser and jitter
- Correct samples/README.txt: the type is detected from the headers
</commit_message>
<xml_diff>
--- a/samples/a_r_25_out.xlsx
+++ b/samples/a_r_25_out.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח נוכחות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="דוח נוכחות" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,15 +43,10 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00990000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -65,7 +60,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCCCC"/>
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -105,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -119,13 +119,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -606,7 +609,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -616,60 +619,52 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>7.97</t>
+          <t>7.35</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="L5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>02/02/2023</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>יום חמישי</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>08:09</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>16:07</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>7.97</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>07:57</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>7.52</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -685,12 +680,12 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -700,60 +695,52 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>7.42</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="4" t="inlineStr"/>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="L7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>07/02/2023</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>יום שלישי</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>07:58</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>15:50</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>7.87</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr"/>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>08:05</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>7.38</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr"/>
+      <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -769,12 +756,12 @@
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>08:04</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -784,60 +771,52 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>8.12</t>
+          <t>7.52</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr"/>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="L9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>13/02/2023</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>יום שני</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>07:55</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>14:52</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>6.95</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=6.50 computed=7.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>08:02</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>6.53</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -853,12 +832,12 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>08:05</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -868,60 +847,52 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>7.75</t>
+          <t>7.65</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="L11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>15/02/2023</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>יום רביעי</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>08:29</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>16:36</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>8.12</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>7.52</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr"/>
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr"/>
+      <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -937,12 +908,12 @@
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -952,60 +923,52 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>7.47</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr"/>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="L13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>19/02/2023</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>יום ראשון</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>08:06</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>15:54</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>7.80</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="C14" s="5" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>08:03</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>7.40</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr"/>
+      <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr"/>
+      <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1021,12 +984,12 @@
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>07:52</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1036,60 +999,52 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>8.22</t>
+          <t>7.37</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr"/>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="L15" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>22/02/2023</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>יום רביעי</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>08:08</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>16:04</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>7.93</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="C16" s="5" t="inlineStr"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>08:02</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>7.43</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr"/>
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1105,12 +1060,12 @@
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1120,60 +1075,52 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>7.05</t>
+          <t>6.63</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr"/>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=6.50 computed=7.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="L17" s="4" t="inlineStr"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>26/02/2023</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>יום ראשון</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>07:58</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>16:08</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>8.17</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>7.57</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1189,12 +1136,12 @@
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>08:10</t>
+          <t>08:04</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1204,122 +1151,118 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>7.73</t>
+          <t>7.42</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="4" t="inlineStr"/>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>daily_hours mismatch: declared=7.50 computed=8.00 diff=0.50</t>
-        </is>
-      </c>
+      <c r="L19" s="4" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr"/>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>117.88</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr"/>
-      <c r="K20" s="5" t="inlineStr"/>
-      <c r="L20" s="5" t="inlineStr"/>
+      <c r="B20" s="6" t="inlineStr"/>
+      <c r="C20" s="6" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>110.18</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>ימים</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B22" s="8" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>סה"כ שעות</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>117.88</t>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>110.18</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>100% שעות</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>117.88</t>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>110.18</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>125% שעות</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>150% שעות</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n">
+      <c r="B26" s="8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>150% שבת</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n">
+      <c r="B27" s="8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>בונוס</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n">
+      <c r="B28" s="8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>נסיעות</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n">
+      <c r="B29" s="8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Read scanned timesheets cell by cell
- New src/readers/table_ocr.py: deskew the page, find the table by its
  ruling lines, read each column with a per-column character whitelist,
  then fix dates from their neighbours and times so out - in == hours
- Use it for Type-A reports (PDFReader(read_tables=True)); Type B unchanged
- Parse the summary block when OCR reads סה"כ with stray marks
- Recompute monthly hours and payment from the jittered hours
- Replace the parser's print() debugging with logger.debug
- Add unit tests and an end-to-end test against a hand transcription
</commit_message>
<xml_diff>
--- a/samples/a_r_25_out.xlsx
+++ b/samples/a_r_25_out.xlsx
@@ -604,12 +604,12 @@
       <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>08:05</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>7.35</t>
+          <t>7.58</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
@@ -642,12 +642,12 @@
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>07:57</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>7.52</t>
+          <t>7.40</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr"/>
@@ -680,12 +680,12 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>08:02</t>
+          <t>07:57</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>7.42</t>
+          <t>7.58</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
@@ -718,7 +718,7 @@
       <c r="C8" s="5" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>08:05</t>
+          <t>07:57</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>7.38</t>
+          <t>7.52</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr"/>
@@ -756,12 +756,12 @@
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>08:04</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -794,7 +794,7 @@
       <c r="C10" s="5" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>08:02</t>
+          <t>08:04</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>6.53</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr"/>
@@ -832,12 +832,12 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>7.65</t>
+          <t>7.48</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
@@ -870,12 +870,12 @@
       <c r="C12" s="5" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>16:29</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>7.52</t>
+          <t>7.38</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr"/>
@@ -913,7 +913,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>7.47</t>
+          <t>7.53</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
@@ -946,12 +946,12 @@
       <c r="C14" s="5" t="inlineStr"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>7.40</t>
+          <t>7.33</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr"/>
@@ -984,12 +984,12 @@
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>08:05</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>7.37</t>
+          <t>7.63</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
@@ -1022,12 +1022,12 @@
       <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>08:02</t>
+          <t>08:04</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>7.43</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr"/>
@@ -1060,12 +1060,12 @@
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>07:56</t>
+          <t>08:04</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>6.63</t>
+          <t>6.40</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>7.57</t>
+          <t>7.45</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr"/>
@@ -1136,12 +1136,12 @@
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>08:04</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>7.42</t>
+          <t>7.53</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
@@ -1173,7 +1173,7 @@
       <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>110.18</t>
+          <t>110.33</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr"/>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>110.18</t>
+          <t>110.33</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>110.18</t>
+          <t>110.33</t>
         </is>
       </c>
     </row>

</xml_diff>